<commit_message>
new updates with 25
</commit_message>
<xml_diff>
--- a/data/fr/FR_Budget_Status.xlsx
+++ b/data/fr/FR_Budget_Status.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\WR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{580F48C6-7F06-436C-A2E2-C1C44CFF7059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020"/>
   </bookViews>
   <sheets>
     <sheet name="OPEN LINE FR" sheetId="1" r:id="rId1"/>
@@ -19,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'OPEN LINE FR'!$A$1:$Z$25</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="47">
   <si>
     <t>Plan Head</t>
   </si>
@@ -169,10 +168,43 @@
     <t>SBA (2026-27)</t>
   </si>
   <si>
-    <t>SBA 2025-26</t>
+    <t>SBA 2026-27</t>
   </si>
   <si>
-    <t>SBA 2026-27</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                                                                                                              </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Actual.  Expenditure of Demand 16 upto as on  25.09.2026  (Fig.in Thousand) </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                                                                                                                                       </t>
+    </r>
   </si>
   <si>
     <r>
@@ -196,7 +228,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Actual.  Expenditure of Demand 16 GSU as on  05.09.2026  (Fig.in Thousand)</t>
+      <t>Actual.  Expenditure of Demand 16 GSU as on  25.09.2026  (Fig.in Thousand)</t>
     </r>
     <r>
       <rPr>
@@ -210,47 +242,11 @@
       <t xml:space="preserve">                                                                                                             </t>
     </r>
   </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">                                                                                                              </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Actual.  Expenditure of Demand 16 upto as on  05.09.2026  (Fig.in Thousand) </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">                                                                                                                                       </t>
-    </r>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1512,7 +1508,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1603,10 +1599,34 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1618,17 +1638,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1065">
@@ -2693,9 +2707,9 @@
     <cellStyle name="Hyperlink" xfId="1061" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1063" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000025040000}"/>
-    <cellStyle name="Normal 2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000026040000}"/>
-    <cellStyle name="Normal 3" xfId="4" xr:uid="{00000000-0005-0000-0000-000027040000}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2 2" xfId="3"/>
+    <cellStyle name="Normal 3" xfId="4"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2712,9 +2726,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2752,9 +2766,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2789,7 +2803,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2824,7 +2838,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2997,7 +3011,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3031,161 +3045,161 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:244" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="36"/>
-      <c r="T1" s="36"/>
-      <c r="U1" s="36"/>
-      <c r="V1" s="36"/>
-      <c r="W1" s="36"/>
-      <c r="X1" s="36"/>
-      <c r="Y1" s="36"/>
-      <c r="Z1" s="36"/>
-      <c r="AA1" s="36"/>
+      <c r="A1" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="37"/>
+      <c r="T1" s="37"/>
+      <c r="U1" s="37"/>
+      <c r="V1" s="37"/>
+      <c r="W1" s="37"/>
+      <c r="X1" s="37"/>
+      <c r="Y1" s="37"/>
+      <c r="Z1" s="37"/>
+      <c r="AA1" s="37"/>
     </row>
     <row r="2" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="40" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="40" t="s">
+      <c r="A2" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="39"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="37" t="s">
+      <c r="D2" s="40"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="39"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="37" t="s">
+      <c r="G2" s="40"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="39"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="37" t="s">
+      <c r="J2" s="40"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="M2" s="39"/>
-      <c r="N2" s="38"/>
-      <c r="O2" s="37" t="s">
+      <c r="M2" s="40"/>
+      <c r="N2" s="39"/>
+      <c r="O2" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="P2" s="39"/>
-      <c r="Q2" s="38"/>
-      <c r="R2" s="37" t="s">
+      <c r="P2" s="40"/>
+      <c r="Q2" s="39"/>
+      <c r="R2" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="S2" s="39"/>
-      <c r="T2" s="38"/>
-      <c r="U2" s="37" t="s">
+      <c r="S2" s="40"/>
+      <c r="T2" s="39"/>
+      <c r="U2" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="V2" s="39"/>
-      <c r="W2" s="38"/>
-      <c r="X2" s="34" t="s">
+      <c r="V2" s="40"/>
+      <c r="W2" s="39"/>
+      <c r="X2" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="Y2" s="34"/>
-      <c r="Z2" s="34"/>
-      <c r="AA2" s="34"/>
+      <c r="Y2" s="35"/>
+      <c r="Z2" s="35"/>
+      <c r="AA2" s="35"/>
     </row>
     <row r="3" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="41"/>
-      <c r="B3" s="41"/>
-      <c r="C3" s="2" t="s">
+      <c r="A3" s="42"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="M3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="P3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S3" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T3" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="U3" s="2" t="s">
+      <c r="U3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="V3" s="5" t="s">
+      <c r="V3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="W3" s="2" t="s">
+      <c r="W3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="X3" s="2" t="s">
+      <c r="X3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="Y3" s="5" t="s">
+      <c r="Y3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="Z3" s="2" t="s">
+      <c r="Z3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="AA3" s="5" t="s">
+      <c r="AA3" s="12" t="s">
         <v>37</v>
       </c>
     </row>
@@ -3200,11 +3214,11 @@
         <v>146190</v>
       </c>
       <c r="D4" s="13">
-        <v>77298</v>
+        <v>80861</v>
       </c>
       <c r="E4" s="14">
         <f>D4-C4</f>
-        <v>-68892</v>
+        <v>-65329</v>
       </c>
       <c r="F4" s="11">
         <v>0</v>
@@ -3252,7 +3266,7 @@
       <c r="S4" s="14">
         <v>0</v>
       </c>
-      <c r="T4" s="7">
+      <c r="T4" s="14">
         <f t="shared" ref="T4:T7" si="1">S4-R4</f>
         <v>0</v>
       </c>
@@ -3272,15 +3286,15 @@
       </c>
       <c r="Y4" s="13">
         <f t="shared" si="3"/>
-        <v>77992</v>
+        <v>81555</v>
       </c>
       <c r="Z4" s="14">
         <f>Y4-X4</f>
-        <v>-82911</v>
-      </c>
-      <c r="AA4" s="6">
+        <v>-79348</v>
+      </c>
+      <c r="AA4" s="13">
         <f>Y4/X4*100</f>
-        <v>48.471439314369526</v>
+        <v>50.685816920753503</v>
       </c>
       <c r="AB4"/>
       <c r="AC4"/>
@@ -3357,36 +3371,36 @@
       <c r="CV4"/>
     </row>
     <row r="5" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="A5" s="3">
         <v>1700</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="11">
         <v>4107</v>
       </c>
-      <c r="D5" s="6">
-        <v>7690</v>
+      <c r="D5" s="13">
+        <v>8656</v>
       </c>
       <c r="E5" s="14">
         <f t="shared" ref="E5:E21" si="4">D5-C5</f>
-        <v>3583</v>
-      </c>
-      <c r="F5" s="5">
+        <v>4549</v>
+      </c>
+      <c r="F5" s="12">
         <v>14120</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="3">
         <v>864</v>
       </c>
       <c r="H5" s="14">
         <f t="shared" si="0"/>
         <v>-13256</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="12">
         <v>14000</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="13">
         <v>3247</v>
       </c>
       <c r="K5" s="14">
@@ -3399,34 +3413,34 @@
       <c r="M5" s="14">
         <v>0</v>
       </c>
-      <c r="N5" s="7">
+      <c r="N5" s="14">
         <f t="shared" ref="N5:N21" si="6">M5-L5</f>
         <v>0</v>
       </c>
-      <c r="O5" s="7">
-        <v>0</v>
-      </c>
-      <c r="P5" s="8">
+      <c r="O5" s="14">
+        <v>0</v>
+      </c>
+      <c r="P5" s="15">
         <v>0</v>
       </c>
       <c r="Q5" s="14">
         <f t="shared" ref="Q5:Q21" si="7">P5-O5</f>
         <v>0</v>
       </c>
-      <c r="R5" s="7">
-        <v>0</v>
-      </c>
-      <c r="S5" s="7">
-        <v>0</v>
-      </c>
-      <c r="T5" s="7">
+      <c r="R5" s="14">
+        <v>0</v>
+      </c>
+      <c r="S5" s="14">
+        <v>0</v>
+      </c>
+      <c r="T5" s="14">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="U5" s="5">
-        <v>0</v>
-      </c>
-      <c r="V5" s="6">
+      <c r="U5" s="12">
+        <v>0</v>
+      </c>
+      <c r="V5" s="13">
         <v>0</v>
       </c>
       <c r="W5" s="14">
@@ -3439,73 +3453,73 @@
       </c>
       <c r="Y5" s="13">
         <f t="shared" si="3"/>
-        <v>11801</v>
+        <v>12767</v>
       </c>
       <c r="Z5" s="14">
         <f t="shared" ref="Z5:Z21" si="8">Y5-X5</f>
-        <v>-20426</v>
-      </c>
-      <c r="AA5" s="6">
+        <v>-19460</v>
+      </c>
+      <c r="AA5" s="13">
         <f t="shared" ref="AA5:AA20" si="9">Y5/X5*100</f>
-        <v>36.618363484035129</v>
+        <v>39.615850063611255</v>
       </c>
     </row>
     <row r="6" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+      <c r="A6" s="3">
         <v>2900</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="2">
-        <v>0</v>
-      </c>
-      <c r="D6" s="6">
+      <c r="C6" s="11">
+        <v>0</v>
+      </c>
+      <c r="D6" s="13">
         <v>0</v>
       </c>
       <c r="E6" s="14">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="F6" s="5">
-        <v>0</v>
-      </c>
-      <c r="G6" s="6">
+      <c r="F6" s="12">
+        <v>0</v>
+      </c>
+      <c r="G6" s="13">
         <v>0</v>
       </c>
       <c r="H6" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I6" s="5">
-        <v>0</v>
-      </c>
-      <c r="J6" s="6">
+      <c r="I6" s="12">
+        <v>0</v>
+      </c>
+      <c r="J6" s="13">
         <v>0</v>
       </c>
       <c r="K6" s="14">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="14">
         <v>0</v>
       </c>
       <c r="M6" s="14">
         <v>0</v>
       </c>
-      <c r="N6" s="7">
+      <c r="N6" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O6" s="7">
+      <c r="O6" s="14">
         <v>120318</v>
       </c>
-      <c r="P6" s="8">
-        <v>57289</v>
+      <c r="P6" s="15">
+        <v>64676</v>
       </c>
       <c r="Q6" s="14">
         <f t="shared" si="7"/>
-        <v>-63029</v>
+        <v>-55642</v>
       </c>
       <c r="R6" s="14">
         <v>0</v>
@@ -3513,14 +3527,14 @@
       <c r="S6" s="14">
         <v>0</v>
       </c>
-      <c r="T6" s="7">
+      <c r="T6" s="14">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="U6" s="5">
-        <v>0</v>
-      </c>
-      <c r="V6" s="6">
+      <c r="U6" s="12">
+        <v>0</v>
+      </c>
+      <c r="V6" s="13">
         <v>0</v>
       </c>
       <c r="W6" s="14">
@@ -3533,48 +3547,48 @@
       </c>
       <c r="Y6" s="13">
         <f t="shared" si="3"/>
-        <v>57289</v>
+        <v>64676</v>
       </c>
       <c r="Z6" s="14">
         <f t="shared" si="8"/>
-        <v>-63029</v>
-      </c>
-      <c r="AA6" s="6">
+        <v>-55642</v>
+      </c>
+      <c r="AA6" s="13">
         <f t="shared" si="9"/>
-        <v>47.614654498911221</v>
+        <v>53.754217988995819</v>
       </c>
     </row>
     <row r="7" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+      <c r="A7" s="3">
         <v>3000</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="2">
-        <v>0</v>
-      </c>
-      <c r="D7" s="6">
+      <c r="C7" s="11">
+        <v>0</v>
+      </c>
+      <c r="D7" s="13">
         <v>0</v>
       </c>
       <c r="E7" s="14">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="F7" s="5">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6">
+      <c r="F7" s="12">
+        <v>0</v>
+      </c>
+      <c r="G7" s="13">
         <v>0</v>
       </c>
       <c r="H7" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I7" s="5">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6">
+      <c r="I7" s="12">
+        <v>0</v>
+      </c>
+      <c r="J7" s="13">
         <v>0</v>
       </c>
       <c r="K7" s="14">
@@ -3587,34 +3601,34 @@
       <c r="M7" s="14">
         <v>0</v>
       </c>
-      <c r="N7" s="7">
+      <c r="N7" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O7" s="7">
+      <c r="O7" s="14">
         <v>316420</v>
       </c>
-      <c r="P7" s="8">
-        <v>254179</v>
+      <c r="P7" s="15">
+        <v>269444</v>
       </c>
       <c r="Q7" s="14">
         <f t="shared" si="7"/>
-        <v>-62241</v>
-      </c>
-      <c r="R7" s="7">
-        <v>0</v>
-      </c>
-      <c r="S7" s="7">
-        <v>0</v>
-      </c>
-      <c r="T7" s="7">
+        <v>-46976</v>
+      </c>
+      <c r="R7" s="14">
+        <v>0</v>
+      </c>
+      <c r="S7" s="14">
+        <v>0</v>
+      </c>
+      <c r="T7" s="14">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="U7" s="5">
+      <c r="U7" s="12">
         <v>191000</v>
       </c>
-      <c r="V7" s="6">
+      <c r="V7" s="13">
         <v>109758</v>
       </c>
       <c r="W7" s="14">
@@ -3627,48 +3641,48 @@
       </c>
       <c r="Y7" s="13">
         <f t="shared" si="3"/>
-        <v>363937</v>
+        <v>379202</v>
       </c>
       <c r="Z7" s="14">
         <f t="shared" si="8"/>
-        <v>-143483</v>
-      </c>
-      <c r="AA7" s="6">
+        <v>-128218</v>
+      </c>
+      <c r="AA7" s="13">
         <f t="shared" si="9"/>
-        <v>71.723030231366522</v>
+        <v>74.73138622837098</v>
       </c>
     </row>
     <row r="8" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>3100</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="2">
-        <v>0</v>
-      </c>
-      <c r="D8" s="6">
+      <c r="C8" s="11">
+        <v>0</v>
+      </c>
+      <c r="D8" s="13">
         <v>0</v>
       </c>
       <c r="E8" s="14">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="F8" s="5">
-        <v>0</v>
-      </c>
-      <c r="G8" s="6">
+      <c r="F8" s="12">
+        <v>0</v>
+      </c>
+      <c r="G8" s="13">
         <v>0</v>
       </c>
       <c r="H8" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I8" s="5">
-        <v>0</v>
-      </c>
-      <c r="J8" s="6">
+      <c r="I8" s="12">
+        <v>0</v>
+      </c>
+      <c r="J8" s="13">
         <v>0</v>
       </c>
       <c r="K8" s="14">
@@ -3681,39 +3695,39 @@
       <c r="M8" s="14">
         <v>0</v>
       </c>
-      <c r="N8" s="7">
+      <c r="N8" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O8" s="7">
+      <c r="O8" s="14">
         <v>2645397</v>
       </c>
-      <c r="P8" s="8">
-        <v>3406763</v>
+      <c r="P8" s="15">
+        <v>3459926</v>
       </c>
       <c r="Q8" s="14">
         <f t="shared" si="7"/>
-        <v>761366</v>
-      </c>
-      <c r="R8" s="7">
-        <v>0</v>
-      </c>
-      <c r="S8" s="7">
-        <v>0</v>
-      </c>
-      <c r="T8" s="7">
+        <v>814529</v>
+      </c>
+      <c r="R8" s="14">
+        <v>0</v>
+      </c>
+      <c r="S8" s="14">
+        <v>0</v>
+      </c>
+      <c r="T8" s="14">
         <f t="shared" ref="T8:T13" si="10">S8-R8</f>
         <v>0</v>
       </c>
-      <c r="U8" s="5">
+      <c r="U8" s="12">
         <v>317398</v>
       </c>
-      <c r="V8" s="6">
-        <v>285936</v>
+      <c r="V8" s="13">
+        <v>345939</v>
       </c>
       <c r="W8" s="14">
         <f t="shared" si="2"/>
-        <v>-31462</v>
+        <v>28541</v>
       </c>
       <c r="X8" s="12">
         <f t="shared" si="3"/>
@@ -3721,15 +3735,15 @@
       </c>
       <c r="Y8" s="13">
         <f t="shared" si="3"/>
-        <v>3692699</v>
+        <v>3805865</v>
       </c>
       <c r="Z8" s="14">
         <f t="shared" si="8"/>
-        <v>729904</v>
-      </c>
-      <c r="AA8" s="6">
+        <v>843070</v>
+      </c>
+      <c r="AA8" s="13">
         <f t="shared" si="9"/>
-        <v>124.63565653377975</v>
+        <v>128.45522555559867</v>
       </c>
     </row>
     <row r="9" spans="1:244" s="4" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3783,11 +3797,11 @@
         <v>35380</v>
       </c>
       <c r="P9" s="15">
-        <v>27875</v>
+        <v>50862</v>
       </c>
       <c r="Q9" s="14">
         <f t="shared" si="7"/>
-        <v>-7505</v>
+        <v>15482</v>
       </c>
       <c r="R9" s="14">
         <v>0</v>
@@ -3803,11 +3817,11 @@
         <v>96867</v>
       </c>
       <c r="V9" s="13">
-        <v>123322</v>
+        <v>133076</v>
       </c>
       <c r="W9" s="14">
         <f t="shared" si="2"/>
-        <v>26455</v>
+        <v>36209</v>
       </c>
       <c r="X9" s="12">
         <f t="shared" si="3"/>
@@ -3815,15 +3829,15 @@
       </c>
       <c r="Y9" s="13">
         <f t="shared" si="3"/>
-        <v>151197</v>
+        <v>183938</v>
       </c>
       <c r="Z9" s="14">
         <f t="shared" si="8"/>
-        <v>18930</v>
-      </c>
-      <c r="AA9" s="6">
+        <v>51671</v>
+      </c>
+      <c r="AA9" s="13">
         <f t="shared" si="9"/>
-        <v>114.31195989929461</v>
+        <v>139.06567775786854</v>
       </c>
       <c r="AB9"/>
       <c r="AC9"/>
@@ -4054,11 +4068,11 @@
         <v>159700</v>
       </c>
       <c r="D10" s="13">
-        <v>10447</v>
+        <v>19998</v>
       </c>
       <c r="E10" s="14">
         <f t="shared" si="4"/>
-        <v>-149253</v>
+        <v>-139702</v>
       </c>
       <c r="F10" s="12">
         <v>0</v>
@@ -4070,7 +4084,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="12">
         <v>0</v>
       </c>
       <c r="J10" s="13">
@@ -4100,13 +4114,13 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="R10" s="7">
-        <v>0</v>
-      </c>
-      <c r="S10" s="7">
-        <v>0</v>
-      </c>
-      <c r="T10" s="7">
+      <c r="R10" s="14">
+        <v>0</v>
+      </c>
+      <c r="S10" s="14">
+        <v>0</v>
+      </c>
+      <c r="T10" s="14">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
@@ -4114,11 +4128,11 @@
         <v>363143</v>
       </c>
       <c r="V10" s="13">
-        <v>112591</v>
+        <v>120409</v>
       </c>
       <c r="W10" s="14">
         <f t="shared" si="2"/>
-        <v>-250552</v>
+        <v>-242734</v>
       </c>
       <c r="X10" s="12">
         <f t="shared" si="3"/>
@@ -4126,15 +4140,15 @@
       </c>
       <c r="Y10" s="13">
         <f t="shared" si="3"/>
-        <v>123038</v>
+        <v>140407</v>
       </c>
       <c r="Z10" s="14">
         <f t="shared" si="8"/>
-        <v>-399805</v>
-      </c>
-      <c r="AA10" s="6">
+        <v>-382436</v>
+      </c>
+      <c r="AA10" s="13">
         <f t="shared" si="9"/>
-        <v>23.532494458183432</v>
+        <v>26.854524207075549</v>
       </c>
       <c r="AB10"/>
       <c r="AC10"/>
@@ -4355,36 +4369,36 @@
       <c r="IJ10"/>
     </row>
     <row r="11" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
+      <c r="A11" s="3">
         <v>3600</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="11">
         <v>174056</v>
       </c>
-      <c r="D11" s="6">
-        <v>78354</v>
+      <c r="D11" s="13">
+        <v>84377</v>
       </c>
       <c r="E11" s="14">
         <f t="shared" si="4"/>
-        <v>-95702</v>
-      </c>
-      <c r="F11" s="5">
-        <v>0</v>
-      </c>
-      <c r="G11" s="6">
+        <v>-89679</v>
+      </c>
+      <c r="F11" s="12">
+        <v>0</v>
+      </c>
+      <c r="G11" s="13">
         <v>0</v>
       </c>
       <c r="H11" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="12">
         <v>25830</v>
       </c>
-      <c r="J11" s="6">
+      <c r="J11" s="13">
         <v>0</v>
       </c>
       <c r="K11" s="14">
@@ -4397,7 +4411,7 @@
       <c r="M11" s="14">
         <v>0</v>
       </c>
-      <c r="N11" s="7">
+      <c r="N11" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -4411,25 +4425,25 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="R11" s="7">
-        <v>0</v>
-      </c>
-      <c r="S11" s="7">
-        <v>0</v>
-      </c>
-      <c r="T11" s="7">
+      <c r="R11" s="14">
+        <v>0</v>
+      </c>
+      <c r="S11" s="14">
+        <v>0</v>
+      </c>
+      <c r="T11" s="14">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="U11" s="5">
+      <c r="U11" s="12">
         <v>107957</v>
       </c>
-      <c r="V11" s="6">
-        <v>16570</v>
+      <c r="V11" s="13">
+        <v>20718</v>
       </c>
       <c r="W11" s="14">
         <f t="shared" si="2"/>
-        <v>-91387</v>
+        <v>-87239</v>
       </c>
       <c r="X11" s="12">
         <f t="shared" si="3"/>
@@ -4437,61 +4451,61 @@
       </c>
       <c r="Y11" s="13">
         <f t="shared" si="3"/>
-        <v>94924</v>
+        <v>105095</v>
       </c>
       <c r="Z11" s="14">
         <f t="shared" si="8"/>
-        <v>-212919</v>
-      </c>
-      <c r="AA11" s="6">
+        <v>-202748</v>
+      </c>
+      <c r="AA11" s="13">
         <f t="shared" si="9"/>
-        <v>30.835198461553453</v>
+        <v>34.139155348667991</v>
       </c>
     </row>
     <row r="12" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+      <c r="A12" s="3">
         <v>3700</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="2">
-        <v>0</v>
-      </c>
-      <c r="D12" s="6">
+      <c r="C12" s="11">
+        <v>0</v>
+      </c>
+      <c r="D12" s="13">
         <v>0</v>
       </c>
       <c r="E12" s="14">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="F12" s="2">
-        <v>0</v>
-      </c>
-      <c r="G12" s="6">
+      <c r="F12" s="11">
+        <v>0</v>
+      </c>
+      <c r="G12" s="13">
         <v>0</v>
       </c>
       <c r="H12" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I12" s="5">
-        <v>0</v>
-      </c>
-      <c r="J12" s="6">
+      <c r="I12" s="12">
+        <v>0</v>
+      </c>
+      <c r="J12" s="13">
         <v>0</v>
       </c>
       <c r="K12" s="14">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L12" s="7">
+      <c r="L12" s="14">
         <v>0</v>
       </c>
       <c r="M12" s="14">
         <v>0</v>
       </c>
-      <c r="N12" s="7">
+      <c r="N12" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -4505,20 +4519,20 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="R12" s="7">
-        <v>0</v>
-      </c>
-      <c r="S12" s="7">
-        <v>0</v>
-      </c>
-      <c r="T12" s="7">
+      <c r="R12" s="14">
+        <v>0</v>
+      </c>
+      <c r="S12" s="14">
+        <v>0</v>
+      </c>
+      <c r="T12" s="14">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="U12" s="5">
-        <v>0</v>
-      </c>
-      <c r="V12" s="6">
+      <c r="U12" s="12">
+        <v>0</v>
+      </c>
+      <c r="V12" s="13">
         <v>0</v>
       </c>
       <c r="W12" s="14">
@@ -4537,42 +4551,42 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="AA12" s="6" t="e">
+      <c r="AA12" s="13" t="e">
         <f t="shared" si="9"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="13" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
+      <c r="A13" s="3">
         <v>4100</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="6">
-        <v>10884</v>
-      </c>
-      <c r="D13" s="6">
-        <v>22627</v>
+      <c r="C13" s="12">
+        <v>38062</v>
+      </c>
+      <c r="D13" s="13">
+        <v>24345</v>
       </c>
       <c r="E13" s="14">
         <f t="shared" si="4"/>
-        <v>11743</v>
-      </c>
-      <c r="F13" s="5">
+        <v>-13717</v>
+      </c>
+      <c r="F13" s="12">
         <v>1</v>
       </c>
-      <c r="G13" s="6">
+      <c r="G13" s="13">
         <v>0</v>
       </c>
       <c r="H13" s="14">
         <f t="shared" si="0"/>
         <v>-1</v>
       </c>
-      <c r="I13" s="5">
+      <c r="I13" s="12">
         <v>309</v>
       </c>
-      <c r="J13" s="6">
+      <c r="J13" s="13">
         <v>0</v>
       </c>
       <c r="K13" s="14">
@@ -4585,7 +4599,7 @@
       <c r="M13" s="14">
         <v>0</v>
       </c>
-      <c r="N13" s="7">
+      <c r="N13" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -4599,20 +4613,20 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="R13" s="7">
-        <v>0</v>
-      </c>
-      <c r="S13" s="7">
-        <v>0</v>
-      </c>
-      <c r="T13" s="7">
+      <c r="R13" s="14">
+        <v>0</v>
+      </c>
+      <c r="S13" s="14">
+        <v>0</v>
+      </c>
+      <c r="T13" s="14">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="U13" s="5">
+      <c r="U13" s="12">
         <v>2000</v>
       </c>
-      <c r="V13" s="6">
+      <c r="V13" s="13">
         <v>1646</v>
       </c>
       <c r="W13" s="14">
@@ -4621,52 +4635,52 @@
       </c>
       <c r="X13" s="12">
         <f t="shared" si="3"/>
-        <v>13194</v>
+        <v>40372</v>
       </c>
       <c r="Y13" s="13">
         <f t="shared" si="3"/>
-        <v>24273</v>
+        <v>25991</v>
       </c>
       <c r="Z13" s="14">
         <f t="shared" si="8"/>
-        <v>11079</v>
-      </c>
-      <c r="AA13" s="6">
+        <v>-14381</v>
+      </c>
+      <c r="AA13" s="13">
         <f t="shared" si="9"/>
-        <v>183.9699863574352</v>
+        <v>64.37877737045477</v>
       </c>
     </row>
     <row r="14" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
+      <c r="A14" s="3">
         <v>4200</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="11">
         <v>35702</v>
       </c>
-      <c r="D14" s="6">
-        <v>5129</v>
+      <c r="D14" s="13">
+        <v>5681</v>
       </c>
       <c r="E14" s="14">
         <f t="shared" si="4"/>
-        <v>-30573</v>
-      </c>
-      <c r="F14" s="5">
+        <v>-30021</v>
+      </c>
+      <c r="F14" s="12">
         <v>2000</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="13">
         <v>0</v>
       </c>
       <c r="H14" s="14">
         <f t="shared" si="0"/>
         <v>-2000</v>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="12">
         <v>5000</v>
       </c>
-      <c r="J14" s="6">
+      <c r="J14" s="13">
         <v>0</v>
       </c>
       <c r="K14" s="14">
@@ -4679,7 +4693,7 @@
       <c r="M14" s="14">
         <v>0</v>
       </c>
-      <c r="N14" s="7">
+      <c r="N14" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -4693,20 +4707,20 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="R14" s="7">
-        <v>0</v>
-      </c>
-      <c r="S14" s="7">
-        <v>0</v>
-      </c>
-      <c r="T14" s="7">
+      <c r="R14" s="14">
+        <v>0</v>
+      </c>
+      <c r="S14" s="14">
+        <v>0</v>
+      </c>
+      <c r="T14" s="14">
         <f t="shared" ref="T14:T15" si="11">S14-R14</f>
         <v>0</v>
       </c>
-      <c r="U14" s="5">
+      <c r="U14" s="12">
         <v>11000</v>
       </c>
-      <c r="V14" s="6">
+      <c r="V14" s="13">
         <v>0</v>
       </c>
       <c r="W14" s="14">
@@ -4719,61 +4733,61 @@
       </c>
       <c r="Y14" s="13">
         <f t="shared" si="3"/>
-        <v>5129</v>
+        <v>5681</v>
       </c>
       <c r="Z14" s="14">
         <f t="shared" si="8"/>
-        <v>-48573</v>
-      </c>
-      <c r="AA14" s="6">
+        <v>-48021</v>
+      </c>
+      <c r="AA14" s="13">
         <f t="shared" si="9"/>
-        <v>9.5508547167703259</v>
+        <v>10.578749394808387</v>
       </c>
     </row>
     <row r="15" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+      <c r="A15" s="3">
         <v>5100</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="11">
         <v>62500</v>
       </c>
-      <c r="D15" s="6">
-        <v>50145</v>
+      <c r="D15" s="13">
+        <v>55657</v>
       </c>
       <c r="E15" s="14">
         <f t="shared" si="4"/>
-        <v>-12355</v>
-      </c>
-      <c r="F15" s="5">
+        <v>-6843</v>
+      </c>
+      <c r="F15" s="12">
         <v>12000</v>
       </c>
-      <c r="G15" s="6">
-        <v>5156</v>
+      <c r="G15" s="13">
+        <v>10903</v>
       </c>
       <c r="H15" s="14">
         <f t="shared" si="0"/>
-        <v>-6844</v>
-      </c>
-      <c r="I15" s="5">
+        <v>-1097</v>
+      </c>
+      <c r="I15" s="12">
         <v>23000</v>
       </c>
-      <c r="J15" s="6">
+      <c r="J15" s="13">
         <v>4551</v>
       </c>
       <c r="K15" s="14">
         <f t="shared" si="5"/>
         <v>-18449</v>
       </c>
-      <c r="L15" s="7">
+      <c r="L15" s="14">
         <v>0</v>
       </c>
       <c r="M15" s="14">
         <v>0</v>
       </c>
-      <c r="N15" s="7">
+      <c r="N15" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -4787,20 +4801,20 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="R15" s="7">
-        <v>0</v>
-      </c>
-      <c r="S15" s="7">
-        <v>0</v>
-      </c>
-      <c r="T15" s="7">
+      <c r="R15" s="14">
+        <v>0</v>
+      </c>
+      <c r="S15" s="14">
+        <v>0</v>
+      </c>
+      <c r="T15" s="14">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="U15" s="5">
-        <v>0</v>
-      </c>
-      <c r="V15" s="6">
+      <c r="U15" s="12">
+        <v>0</v>
+      </c>
+      <c r="V15" s="13">
         <v>0</v>
       </c>
       <c r="W15" s="14">
@@ -4813,15 +4827,15 @@
       </c>
       <c r="Y15" s="13">
         <f t="shared" si="3"/>
-        <v>59852</v>
+        <v>71111</v>
       </c>
       <c r="Z15" s="14">
         <f t="shared" si="8"/>
-        <v>-37648</v>
-      </c>
-      <c r="AA15" s="6">
+        <v>-26389</v>
+      </c>
+      <c r="AA15" s="13">
         <f t="shared" si="9"/>
-        <v>61.38666666666667</v>
+        <v>72.934358974358972</v>
       </c>
     </row>
     <row r="16" spans="1:244" s="4" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4835,11 +4849,11 @@
         <v>285610</v>
       </c>
       <c r="D16" s="13">
-        <v>125946</v>
+        <v>142024</v>
       </c>
       <c r="E16" s="14">
         <f t="shared" si="4"/>
-        <v>-159664</v>
+        <v>-143586</v>
       </c>
       <c r="F16" s="12">
         <v>0</v>
@@ -4907,15 +4921,15 @@
       </c>
       <c r="Y16" s="13">
         <f t="shared" si="3"/>
-        <v>131048</v>
+        <v>147126</v>
       </c>
       <c r="Z16" s="14">
         <f t="shared" si="8"/>
-        <v>-179864</v>
-      </c>
-      <c r="AA16" s="6">
+        <v>-163786</v>
+      </c>
+      <c r="AA16" s="13">
         <f t="shared" si="9"/>
-        <v>42.149547138740225</v>
+        <v>47.320785302593663</v>
       </c>
       <c r="AB16"/>
       <c r="AC16"/>
@@ -5010,36 +5024,36 @@
       <c r="DN16"/>
     </row>
     <row r="17" spans="1:1476" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
+      <c r="A17" s="3">
         <v>6200</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="2">
-        <v>0</v>
-      </c>
-      <c r="D17" s="6">
+      <c r="C17" s="11">
+        <v>0</v>
+      </c>
+      <c r="D17" s="13">
         <v>0</v>
       </c>
       <c r="E17" s="14">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="F17" s="5">
-        <v>0</v>
-      </c>
-      <c r="G17" s="6">
+      <c r="F17" s="12">
+        <v>0</v>
+      </c>
+      <c r="G17" s="13">
         <v>0</v>
       </c>
       <c r="H17" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I17" s="5">
-        <v>0</v>
-      </c>
-      <c r="J17" s="6">
+      <c r="I17" s="12">
+        <v>0</v>
+      </c>
+      <c r="J17" s="13">
         <v>0</v>
       </c>
       <c r="K17" s="14">
@@ -5052,7 +5066,7 @@
       <c r="M17" s="14">
         <v>0</v>
       </c>
-      <c r="N17" s="7">
+      <c r="N17" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -5066,20 +5080,20 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="R17" s="7">
-        <v>0</v>
-      </c>
-      <c r="S17" s="7">
+      <c r="R17" s="14">
+        <v>0</v>
+      </c>
+      <c r="S17" s="14">
         <v>0</v>
       </c>
       <c r="T17" s="14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="U17" s="5">
-        <v>0</v>
-      </c>
-      <c r="V17" s="6">
+      <c r="U17" s="12">
+        <v>0</v>
+      </c>
+      <c r="V17" s="13">
         <v>0</v>
       </c>
       <c r="W17" s="14">
@@ -5098,7 +5112,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="AA17" s="6" t="e">
+      <c r="AA17" s="13" t="e">
         <f t="shared" si="9"/>
         <v>#DIV/0!</v>
       </c>
@@ -5114,11 +5128,11 @@
         <v>69550</v>
       </c>
       <c r="D18" s="13">
-        <v>31206</v>
+        <v>35429</v>
       </c>
       <c r="E18" s="14">
         <f t="shared" si="4"/>
-        <v>-38344</v>
+        <v>-34121</v>
       </c>
       <c r="F18" s="12">
         <v>12111</v>
@@ -5174,11 +5188,11 @@
         <v>172069</v>
       </c>
       <c r="V18" s="29">
-        <v>53936</v>
+        <v>58923</v>
       </c>
       <c r="W18" s="14">
         <f t="shared" si="2"/>
-        <v>-118133</v>
+        <v>-113146</v>
       </c>
       <c r="X18" s="12">
         <f t="shared" si="3"/>
@@ -5186,15 +5200,15 @@
       </c>
       <c r="Y18" s="13">
         <f t="shared" si="3"/>
-        <v>103375</v>
+        <v>112585</v>
       </c>
       <c r="Z18" s="14">
         <f t="shared" si="8"/>
-        <v>-212358</v>
-      </c>
-      <c r="AA18" s="6">
+        <v>-203148</v>
+      </c>
+      <c r="AA18" s="13">
         <f>Y18/X18*100</f>
-        <v>32.741271897457665</v>
+        <v>35.658293558164651</v>
       </c>
       <c r="AB18"/>
       <c r="AC18"/>
@@ -6647,34 +6661,34 @@
       <c r="BDT18"/>
     </row>
     <row r="19" spans="1:1476" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="2" t="s">
+      <c r="A19" s="3"/>
+      <c r="B19" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="11">
         <v>64034</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="13">
         <v>0</v>
       </c>
       <c r="E19" s="14">
         <f t="shared" si="4"/>
         <v>-64034</v>
       </c>
-      <c r="F19" s="5">
-        <v>0</v>
-      </c>
-      <c r="G19" s="6">
+      <c r="F19" s="12">
+        <v>0</v>
+      </c>
+      <c r="G19" s="13">
         <v>0</v>
       </c>
       <c r="H19" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I19" s="5">
-        <v>0</v>
-      </c>
-      <c r="J19" s="6">
+      <c r="I19" s="12">
+        <v>0</v>
+      </c>
+      <c r="J19" s="13">
         <v>0</v>
       </c>
       <c r="K19" s="14">
@@ -6687,7 +6701,7 @@
       <c r="M19" s="14">
         <v>0</v>
       </c>
-      <c r="N19" s="7">
+      <c r="N19" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -6701,20 +6715,20 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="R19" s="7">
-        <v>0</v>
-      </c>
-      <c r="S19" s="7">
+      <c r="R19" s="14">
+        <v>0</v>
+      </c>
+      <c r="S19" s="14">
         <v>0</v>
       </c>
       <c r="T19" s="14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="U19" s="5">
-        <v>0</v>
-      </c>
-      <c r="V19" s="10">
+      <c r="U19" s="12">
+        <v>0</v>
+      </c>
+      <c r="V19" s="29">
         <v>0</v>
       </c>
       <c r="W19" s="14">
@@ -6733,42 +6747,42 @@
         <f t="shared" si="8"/>
         <v>-64034</v>
       </c>
-      <c r="AA19" s="6">
+      <c r="AA19" s="13">
         <f>Y19/X19*100</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:1476" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
+      <c r="A20" s="3">
         <v>6500</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="11">
         <v>6000</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="13">
         <v>0</v>
       </c>
       <c r="E20" s="14">
         <f t="shared" si="4"/>
         <v>-6000</v>
       </c>
-      <c r="F20" s="5">
-        <v>0</v>
-      </c>
-      <c r="G20" s="6">
+      <c r="F20" s="12">
+        <v>0</v>
+      </c>
+      <c r="G20" s="13">
         <v>0</v>
       </c>
       <c r="H20" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I20" s="5">
-        <v>0</v>
-      </c>
-      <c r="J20" s="6">
+      <c r="I20" s="12">
+        <v>0</v>
+      </c>
+      <c r="J20" s="13">
         <v>0</v>
       </c>
       <c r="K20" s="14">
@@ -6781,7 +6795,7 @@
       <c r="M20" s="14">
         <v>0</v>
       </c>
-      <c r="N20" s="7">
+      <c r="N20" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -6805,10 +6819,10 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="U20" s="5">
+      <c r="U20" s="12">
         <v>10</v>
       </c>
-      <c r="V20" s="6">
+      <c r="V20" s="13">
         <v>0</v>
       </c>
       <c r="W20" s="14">
@@ -6827,45 +6841,45 @@
         <f t="shared" si="8"/>
         <v>-6010</v>
       </c>
-      <c r="AA20" s="6">
+      <c r="AA20" s="13">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:1476" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="38"/>
-      <c r="C21" s="2">
+      <c r="B21" s="39"/>
+      <c r="C21" s="11">
         <f>SUM(C4:C20)</f>
-        <v>1018353</v>
-      </c>
-      <c r="D21" s="1">
+        <v>1045531</v>
+      </c>
+      <c r="D21" s="3">
         <f>SUM(D4:D20)</f>
-        <v>408842</v>
+        <v>457028</v>
       </c>
       <c r="E21" s="14">
         <f t="shared" si="4"/>
-        <v>-609511</v>
-      </c>
-      <c r="F21" s="2">
+        <v>-588503</v>
+      </c>
+      <c r="F21" s="11">
         <f>SUM(F4:F20)</f>
         <v>40232</v>
       </c>
-      <c r="G21" s="1">
+      <c r="G21" s="3">
         <f>SUM(G4:G20)</f>
-        <v>15491</v>
+        <v>21238</v>
       </c>
       <c r="H21" s="14">
         <f t="shared" si="0"/>
-        <v>-24741</v>
-      </c>
-      <c r="I21" s="2">
+        <v>-18994</v>
+      </c>
+      <c r="I21" s="11">
         <f>SUM(I4:I20)</f>
         <v>130592</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="3">
         <f>SUM(J4:J20)</f>
         <v>18459</v>
       </c>
@@ -6873,69 +6887,69 @@
         <f t="shared" si="5"/>
         <v>-112133</v>
       </c>
-      <c r="L21" s="2">
+      <c r="L21" s="11">
         <f>SUM(L4:L20)</f>
         <v>0</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="11">
         <f>SUM(M4:M20)</f>
         <v>0</v>
       </c>
-      <c r="N21" s="7">
+      <c r="N21" s="14">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O21" s="1">
+      <c r="O21" s="3">
         <f>SUM(O4:O20)</f>
         <v>3117515</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="3">
         <f>SUM(P4:P20)</f>
-        <v>3746106</v>
+        <v>3844908</v>
       </c>
       <c r="Q21" s="14">
         <f t="shared" si="7"/>
-        <v>628591</v>
-      </c>
-      <c r="R21" s="1">
+        <v>727393</v>
+      </c>
+      <c r="R21" s="3">
         <f>SUM(R4:R20)</f>
         <v>0</v>
       </c>
-      <c r="S21" s="1">
+      <c r="S21" s="3">
         <f>SUM(S4:S20)</f>
         <v>0</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="3">
         <f>SUM(T4:T20)</f>
         <v>0</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="11">
         <f>SUM(U4:U20)</f>
         <v>1301009</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="3">
         <f>SUM(V4:V20)</f>
-        <v>707656</v>
-      </c>
-      <c r="W21" s="7">
+        <v>794366</v>
+      </c>
+      <c r="W21" s="14">
         <f t="shared" si="2"/>
-        <v>-593353</v>
+        <v>-506643</v>
       </c>
       <c r="X21" s="12">
         <f t="shared" si="13"/>
-        <v>5607701</v>
+        <v>5634879</v>
       </c>
       <c r="Y21" s="13">
         <f t="shared" si="13"/>
-        <v>4896554</v>
+        <v>5135999</v>
       </c>
       <c r="Z21" s="14">
         <f t="shared" si="8"/>
-        <v>-711147</v>
-      </c>
-      <c r="AA21" s="6">
+        <v>-498880</v>
+      </c>
+      <c r="AA21" s="13">
         <f>Y21/X21*100</f>
-        <v>87.318385912515666</v>
+        <v>91.146571204102173</v>
       </c>
     </row>
     <row r="22" spans="1:1476" x14ac:dyDescent="0.25">
@@ -7820,7 +7834,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -7834,88 +7848,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
-      <c r="S1" s="42"/>
-      <c r="T1" s="42"/>
-      <c r="U1" s="42"/>
-      <c r="V1" s="42"/>
-      <c r="W1" s="42"/>
-      <c r="X1" s="42"/>
-      <c r="Y1" s="42"/>
-      <c r="Z1" s="42"/>
-      <c r="AA1" s="42"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="43"/>
+      <c r="U1" s="43"/>
+      <c r="V1" s="43"/>
+      <c r="W1" s="43"/>
+      <c r="X1" s="43"/>
+      <c r="Y1" s="43"/>
+      <c r="Z1" s="43"/>
+      <c r="AA1" s="43"/>
     </row>
     <row r="2" spans="1:35" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="41" t="s">
+      <c r="A2" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41" t="s">
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41" t="s">
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41" t="s">
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41" t="s">
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41" t="s">
+      <c r="P2" s="47"/>
+      <c r="Q2" s="47"/>
+      <c r="R2" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="S2" s="41"/>
-      <c r="T2" s="41"/>
-      <c r="U2" s="41" t="s">
+      <c r="S2" s="47"/>
+      <c r="T2" s="47"/>
+      <c r="U2" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="V2" s="41"/>
-      <c r="W2" s="41"/>
-      <c r="X2" s="34" t="s">
+      <c r="V2" s="47"/>
+      <c r="W2" s="47"/>
+      <c r="X2" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="Y2" s="34"/>
-      <c r="Z2" s="34"/>
-      <c r="AA2" s="34"/>
+      <c r="Y2" s="48"/>
+      <c r="Z2" s="48"/>
+      <c r="AA2" s="48"/>
     </row>
     <row r="3" spans="1:35" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="34"/>
-      <c r="B3" s="34"/>
+      <c r="A3" s="48"/>
+      <c r="B3" s="48"/>
       <c r="C3" s="2" t="s">
         <v>44</v>
       </c>
@@ -7926,7 +7940,7 @@
         <v>24</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>23</v>
@@ -7944,7 +7958,7 @@
         <v>24</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="M3" s="5" t="s">
         <v>23</v>
@@ -7953,7 +7967,7 @@
         <v>24</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>23</v>
@@ -7962,7 +7976,7 @@
         <v>24</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S3" s="2" t="s">
         <v>23</v>
@@ -7971,7 +7985,7 @@
         <v>30</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="V3" s="5" t="s">
         <v>23</v>
@@ -7980,7 +7994,7 @@
         <v>24</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Y3" s="5" t="s">
         <v>23</v>
@@ -9132,11 +9146,11 @@
         <v>446600</v>
       </c>
       <c r="D16" s="6">
-        <v>317088</v>
+        <v>366679</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="2"/>
-        <v>-129512</v>
+        <v>-79921</v>
       </c>
       <c r="F16" s="5">
         <v>0</v>
@@ -9204,15 +9218,15 @@
       </c>
       <c r="Y16" s="6">
         <f t="shared" si="7"/>
-        <v>317088</v>
+        <v>366679</v>
       </c>
       <c r="Z16" s="7">
         <f t="shared" si="8"/>
-        <v>-129512</v>
+        <v>-79921</v>
       </c>
       <c r="AA16" s="6">
         <f t="shared" si="11"/>
-        <v>71.000447828034027</v>
+        <v>82.104567845947145</v>
       </c>
     </row>
     <row r="17" spans="1:34" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -9589,21 +9603,21 @@
       </c>
     </row>
     <row r="21" spans="1:34" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="38"/>
+      <c r="B21" s="46"/>
       <c r="C21" s="2">
         <f>SUM(C4:C20)</f>
         <v>451601</v>
       </c>
       <c r="D21" s="1">
         <f>SUM(D4:D20)</f>
-        <v>319136</v>
+        <v>368727</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" ref="E21" si="20">D21-C21</f>
-        <v>-132465</v>
+        <v>-82874</v>
       </c>
       <c r="F21" s="2">
         <f>SUM(F4:F20)</f>
@@ -9682,15 +9696,15 @@
       </c>
       <c r="Y21" s="6">
         <f t="shared" si="7"/>
-        <v>319263</v>
+        <v>368854</v>
       </c>
       <c r="Z21" s="7">
         <f t="shared" si="8"/>
-        <v>-132340</v>
+        <v>-82749</v>
       </c>
       <c r="AA21" s="6">
         <f t="shared" si="11"/>
-        <v>70.695500251326933</v>
+        <v>81.676605336988459</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -9748,32 +9762,32 @@
       </c>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A36" s="36"/>
-      <c r="B36" s="36"/>
-      <c r="C36" s="36"/>
-      <c r="D36" s="36"/>
-      <c r="E36" s="36"/>
-      <c r="F36" s="36"/>
-      <c r="G36" s="36"/>
-      <c r="H36" s="36"/>
-      <c r="I36" s="36"/>
-      <c r="J36" s="36"/>
-      <c r="K36" s="36"/>
-      <c r="L36" s="36"/>
-      <c r="M36" s="36"/>
-      <c r="N36" s="36"/>
-      <c r="O36" s="36"/>
-      <c r="P36" s="36"/>
-      <c r="Q36" s="36"/>
-      <c r="R36" s="36"/>
-      <c r="S36" s="36"/>
-      <c r="T36" s="36"/>
-      <c r="U36" s="36"/>
-      <c r="V36" s="36"/>
-      <c r="W36" s="36"/>
-      <c r="X36" s="36"/>
-      <c r="Y36" s="36"/>
-      <c r="Z36" s="36"/>
+      <c r="A36" s="44"/>
+      <c r="B36" s="44"/>
+      <c r="C36" s="44"/>
+      <c r="D36" s="44"/>
+      <c r="E36" s="44"/>
+      <c r="F36" s="44"/>
+      <c r="G36" s="44"/>
+      <c r="H36" s="44"/>
+      <c r="I36" s="44"/>
+      <c r="J36" s="44"/>
+      <c r="K36" s="44"/>
+      <c r="L36" s="44"/>
+      <c r="M36" s="44"/>
+      <c r="N36" s="44"/>
+      <c r="O36" s="44"/>
+      <c r="P36" s="44"/>
+      <c r="Q36" s="44"/>
+      <c r="R36" s="44"/>
+      <c r="S36" s="44"/>
+      <c r="T36" s="44"/>
+      <c r="U36" s="44"/>
+      <c r="V36" s="44"/>
+      <c r="W36" s="44"/>
+      <c r="X36" s="44"/>
+      <c r="Y36" s="44"/>
+      <c r="Z36" s="44"/>
       <c r="AA36" t="s">
         <v>36</v>
       </c>

</xml_diff>